<commit_message>
feat: UI color improvements - 종료 grey-600, 선생님휴가 bg-gray-100, 보조강사 yellow+orange border+black caret
</commit_message>
<xml_diff>
--- a/public/보조강사 최종배정표.xlsx
+++ b/public/보조강사 최종배정표.xlsx
@@ -318,14 +318,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>보조강사유튜브쇼츠1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>보조강사유튜브쇼츠2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>보조강사컴활용</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -351,6 +343,14 @@
   </si>
   <si>
     <t>취업팀ㅡ오후</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보조강사쇼츠1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보조강사쇼츠2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1018,8 +1018,8 @@
       <c r="E10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>79</v>
+      <c r="F10" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>43</v>
@@ -1033,7 +1033,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>8</v>
@@ -1042,7 +1042,7 @@
         <v>22</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>44</v>
@@ -1056,7 +1056,7 @@
         <v>7</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>9</v>
@@ -1079,7 +1079,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>16</v>
@@ -1102,7 +1102,7 @@
         <v>24</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>17</v>
@@ -1125,7 +1125,7 @@
         <v>25</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>18</v>
@@ -1148,7 +1148,7 @@
         <v>26</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>19</v>
@@ -1171,7 +1171,7 @@
         <v>27</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>20</v>

</xml_diff>